<commit_message>
Daily EOD data and reports for 2026-08-04
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260804.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260804.xlsx
@@ -569,24 +569,24 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>59.74</v>
+        <v>59.75</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>-0.98</v>
+        <v>-0.97</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>-1.61%</t>
+          <t>-1.60%</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
         <v>11065</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>661023.1</v>
+        <v>661133.75</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>-10843.7</v>
+        <v>-10733.05</v>
       </c>
     </row>
     <row r="8">
@@ -677,24 +677,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>127.05</v>
+        <v>127.09</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>2.75</v>
+        <v>2.79</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2.21%</t>
+          <t>2.24%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>508200</v>
+        <v>508360</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>11000</v>
+        <v>11160</v>
       </c>
     </row>
     <row r="12">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>32.815</v>
+        <v>32.82</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.315</v>
+        <v>0.32</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0.97%</t>
+          <t>0.98%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>42265.72</v>
+        <v>42272.16</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>405.72</v>
+        <v>412.16</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1633137.64</v>
+        <v>1633414.73</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>596.84</v>
+        <v>873.9299999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>